<commit_message>
Adiciona apostila de ensino e atualiza documentacao
</commit_message>
<xml_diff>
--- a/CONTROLE DE PERCENTUAIS DE COMISSÃO VR.xlsx
+++ b/CONTROLE DE PERCENTUAIS DE COMISSÃO VR.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="A:\THAIS\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="U:\--2021\07-Comissao VR\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60B8A027-5F15-402A-B8DB-ED452460E840}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB29EC4D-331A-40E0-B4BB-35A739DDE208}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-165" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-870" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="VR ADM ATUAL" sheetId="2" r:id="rId1"/>
@@ -21,7 +21,6 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'VR ADM ATUAL'!$A$1:$G$35</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -1489,7 +1488,7 @@
     <numFmt numFmtId="44" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="&quot;R$&quot;\ #,##0.00"/>
   </numFmts>
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1573,8 +1572,20 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1605,6 +1616,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="23">
     <border>
@@ -1909,13 +1926,14 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="4">
+  <cellStyleXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="44" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="108">
+  <cellXfs count="123">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1970,9 +1988,6 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="9" fontId="3" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2005,23 +2020,11 @@
     <xf numFmtId="10" fontId="3" fillId="2" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="10" fontId="2" fillId="2" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="10" fontId="2" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="10" fontId="3" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="10" fontId="3" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="10" fontId="2" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -2110,9 +2113,6 @@
     <xf numFmtId="10" fontId="3" fillId="0" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2122,11 +2122,71 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="9" fontId="2" fillId="6" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="3" fillId="6" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="2" fillId="5" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="3" fillId="5" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="5" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="2" fillId="5" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="2" fillId="5" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="10" fontId="2" fillId="5" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="3" fillId="5" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="3" fillId="5" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="10" fontId="3" fillId="5" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="4">
+  <cellStyles count="5">
     <cellStyle name="Hiperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Moeda" xfId="3" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="4" xr:uid="{FF561953-5709-4E5C-B155-84A2331BD9C0}"/>
     <cellStyle name="Porcentagem" xfId="2" builtinId="5"/>
   </cellStyles>
   <dxfs count="1">
@@ -2414,599 +2474,621 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="350" row="2">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{DE5A3704-CC1E-4AFC-89EF-F5BBD49ECE60}">
+  <we:reference id="wa200010725" version="1.0.0.1" store="pt-BR" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="WA200010725" version="1.0.0.1" store="WA200010725" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="claude.fileId" value="&quot;ac774c9b-810a-4f48-9f3e-a54bef1fb5b7&quot;"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:H35"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="77.5703125" style="12" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="58.7109375" style="10" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.7109375" style="15" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="77.5546875" style="12" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="58.6640625" style="10" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.6640625" style="15" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="19" style="10" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.7109375" style="12" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="22.7109375" style="10" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="20.140625" style="23" bestFit="1" customWidth="1"/>
-    <col min="8" max="16384" width="9.140625" style="12"/>
+    <col min="5" max="5" width="18.6640625" style="12" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.6640625" style="10" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.109375" style="22" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="9.109375" style="12"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
         <v>90</v>
       </c>
       <c r="B1" s="9" t="s">
         <v>374</v>
       </c>
-      <c r="C1" s="32" t="s">
+      <c r="C1" s="31" t="s">
         <v>382</v>
       </c>
-      <c r="D1" s="32" t="s">
+      <c r="D1" s="31" t="s">
         <v>383</v>
       </c>
-      <c r="E1" s="32" t="s">
+      <c r="E1" s="31" t="s">
         <v>384</v>
       </c>
-      <c r="F1" s="97" t="s">
+      <c r="F1" s="92" t="s">
         <v>385</v>
       </c>
       <c r="G1" s="18" t="s">
         <v>386</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" s="11" t="s">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" s="102" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="21">
+      <c r="B2" s="110">
         <v>0.05</v>
       </c>
-      <c r="C2" s="21">
+      <c r="C2" s="110">
         <v>0.6</v>
       </c>
-      <c r="D2" s="20">
+      <c r="D2" s="107">
         <v>0.6</v>
       </c>
       <c r="E2" s="11"/>
-      <c r="F2" s="98"/>
+      <c r="F2" s="93"/>
       <c r="G2" s="18" t="s">
         <v>392</v>
       </c>
     </row>
-    <row r="3" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
+    <row r="3" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="102" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="31">
+      <c r="B3" s="107">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="C3" s="35">
+      <c r="C3" s="109">
         <v>0.6</v>
       </c>
-      <c r="D3" s="35">
+      <c r="D3" s="109">
         <v>0.6</v>
       </c>
-      <c r="E3" s="27"/>
-      <c r="F3" s="101"/>
-      <c r="G3" s="25" t="s">
+      <c r="E3" s="26"/>
+      <c r="F3" s="96"/>
+      <c r="G3" s="24" t="s">
         <v>388</v>
       </c>
     </row>
-    <row r="4" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
+    <row r="4" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="103" t="s">
         <v>464</v>
       </c>
-      <c r="B4" s="31">
+      <c r="B4" s="30">
         <v>0.05</v>
       </c>
-      <c r="C4" s="35">
+      <c r="C4" s="33">
         <v>0.6</v>
       </c>
-      <c r="D4" s="35"/>
-      <c r="E4" s="27"/>
-      <c r="F4" s="101"/>
-      <c r="G4" s="25"/>
+      <c r="D4" s="33"/>
+      <c r="E4" s="26"/>
+      <c r="F4" s="96"/>
+      <c r="G4" s="24"/>
       <c r="H4" s="3" t="s">
         <v>465</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="11" t="s">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" s="102" t="s">
         <v>391</v>
       </c>
-      <c r="B5" s="20">
+      <c r="B5" s="107">
         <v>0.03</v>
       </c>
-      <c r="C5" s="32">
+      <c r="C5" s="109">
         <v>0.6</v>
       </c>
-      <c r="D5" s="32">
+      <c r="D5" s="109">
         <v>0.6</v>
       </c>
       <c r="E5" s="16"/>
-      <c r="F5" s="97"/>
+      <c r="F5" s="92"/>
       <c r="G5" s="19"/>
     </row>
-    <row r="6" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
+    <row r="6" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="103" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="29">
+      <c r="B6" s="28">
         <v>0.05</v>
       </c>
-      <c r="C6" s="24"/>
-      <c r="D6" s="26"/>
+      <c r="C6" s="23"/>
+      <c r="D6" s="25"/>
       <c r="E6" s="2"/>
-      <c r="F6" s="99"/>
-      <c r="G6" s="25" t="s">
+      <c r="F6" s="94"/>
+      <c r="G6" s="24" t="s">
         <v>388</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" s="11" t="s">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" s="104" t="s">
         <v>15</v>
       </c>
-      <c r="B7" s="13" t="s">
+      <c r="B7" s="105" t="s">
         <v>379</v>
       </c>
-      <c r="C7" s="32"/>
-      <c r="D7" s="32">
+      <c r="C7" s="106"/>
+      <c r="D7" s="106">
         <v>0.7</v>
       </c>
       <c r="E7" s="16"/>
-      <c r="F7" s="97">
+      <c r="F7" s="92">
         <v>0.7</v>
       </c>
       <c r="G7" s="18" t="s">
         <v>392</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8" s="102" t="s">
         <v>375</v>
       </c>
-      <c r="B8" s="21">
+      <c r="B8" s="110">
         <v>0.1</v>
       </c>
-      <c r="C8" s="32"/>
-      <c r="D8" s="32">
+      <c r="C8" s="109"/>
+      <c r="D8" s="109">
         <v>0.7</v>
       </c>
       <c r="E8" s="17"/>
-      <c r="F8" s="100"/>
+      <c r="F8" s="95"/>
       <c r="G8" s="19"/>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" s="102" t="s">
         <v>25</v>
       </c>
-      <c r="B9" s="20">
+      <c r="B9" s="107">
         <v>0.1</v>
       </c>
-      <c r="C9" s="33"/>
-      <c r="D9" s="32">
+      <c r="C9" s="108"/>
+      <c r="D9" s="109">
         <v>0.6</v>
       </c>
-      <c r="E9" s="17"/>
-      <c r="F9" s="97">
+      <c r="E9" s="115"/>
+      <c r="F9" s="121">
         <v>0.6</v>
       </c>
       <c r="G9" s="19"/>
     </row>
-    <row r="10" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
+    <row r="10" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="103" t="s">
         <v>26</v>
       </c>
-      <c r="B10" s="31">
+      <c r="B10" s="30">
         <v>0.1</v>
       </c>
-      <c r="C10" s="35">
+      <c r="C10" s="33">
         <v>0.6</v>
       </c>
-      <c r="D10" s="35">
+      <c r="D10" s="33">
         <v>0.6</v>
       </c>
-      <c r="E10" s="27"/>
-      <c r="F10" s="101"/>
-      <c r="G10" s="28"/>
-    </row>
-    <row r="11" spans="1:8" s="40" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="104" t="s">
+      <c r="E10" s="26"/>
+      <c r="F10" s="96"/>
+      <c r="G10" s="27"/>
+    </row>
+    <row r="11" spans="1:8" s="35" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="117" t="s">
         <v>27</v>
       </c>
-      <c r="B11" s="37" t="s">
+      <c r="B11" s="118" t="s">
         <v>390</v>
       </c>
-      <c r="C11" s="38">
+      <c r="C11" s="119">
         <v>0.6</v>
       </c>
-      <c r="D11" s="38">
+      <c r="D11" s="119">
         <v>0.6</v>
       </c>
-      <c r="E11" s="39"/>
-      <c r="F11" s="102"/>
-      <c r="G11" s="25" t="s">
+      <c r="E11" s="34"/>
+      <c r="F11" s="97"/>
+      <c r="G11" s="24" t="s">
         <v>392</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B12" s="21" t="s">
+      <c r="B12" s="20" t="s">
         <v>381</v>
       </c>
       <c r="C12" s="13"/>
       <c r="D12" s="14"/>
       <c r="E12" s="11"/>
-      <c r="F12" s="98"/>
+      <c r="F12" s="93"/>
       <c r="G12" s="19"/>
     </row>
-    <row r="13" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
+    <row r="13" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="102" t="s">
         <v>376</v>
       </c>
-      <c r="B13" s="29">
+      <c r="B13" s="110">
         <v>0.1</v>
       </c>
-      <c r="C13" s="30"/>
-      <c r="D13" s="35">
+      <c r="C13" s="120"/>
+      <c r="D13" s="109">
         <v>0.6</v>
       </c>
-      <c r="E13" s="30"/>
-      <c r="F13" s="103">
+      <c r="E13" s="120"/>
+      <c r="F13" s="121">
         <v>0.6</v>
       </c>
-      <c r="G13" s="25" t="s">
+      <c r="G13" s="24" t="s">
         <v>392</v>
       </c>
     </row>
-    <row r="14" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B14" s="29">
+      <c r="B14" s="28">
         <v>0.05</v>
       </c>
-      <c r="C14" s="24"/>
-      <c r="D14" s="26"/>
+      <c r="C14" s="23"/>
+      <c r="D14" s="25"/>
       <c r="E14" s="2"/>
-      <c r="F14" s="99"/>
-      <c r="G14" s="25" t="s">
+      <c r="F14" s="94"/>
+      <c r="G14" s="24" t="s">
         <v>388</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" s="2" t="s">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A15" s="102" t="s">
         <v>40</v>
       </c>
-      <c r="B15" s="21">
+      <c r="B15" s="110">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="C15" s="13"/>
-      <c r="D15" s="14"/>
-      <c r="E15" s="11"/>
-      <c r="F15" s="98"/>
-      <c r="G15" s="18" t="s">
+      <c r="C15" s="111"/>
+      <c r="D15" s="112"/>
+      <c r="E15" s="102"/>
+      <c r="F15" s="113"/>
+      <c r="G15" s="114" t="s">
         <v>388</v>
       </c>
     </row>
-    <row r="16" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="2" t="s">
+    <row r="16" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="102" t="s">
         <v>42</v>
       </c>
-      <c r="B16" s="29">
+      <c r="B16" s="110">
         <v>0.1</v>
       </c>
-      <c r="C16" s="27"/>
-      <c r="D16" s="35">
+      <c r="C16" s="115"/>
+      <c r="D16" s="109">
         <v>0.5</v>
       </c>
-      <c r="E16" s="27"/>
-      <c r="F16" s="103">
+      <c r="E16" s="115"/>
+      <c r="F16" s="121">
         <v>0.5</v>
       </c>
-      <c r="G16" s="25" t="s">
+      <c r="G16" s="24" t="s">
         <v>392</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17" s="2" t="s">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A17" s="102" t="s">
         <v>46</v>
       </c>
-      <c r="B17" s="21">
+      <c r="B17" s="110">
         <v>0.1</v>
       </c>
-      <c r="C17" s="13"/>
-      <c r="D17" s="14"/>
+      <c r="C17" s="111"/>
+      <c r="D17" s="112"/>
       <c r="E17" s="11"/>
-      <c r="F17" s="98"/>
+      <c r="F17" s="93"/>
       <c r="G17" s="18" t="s">
         <v>388</v>
       </c>
     </row>
-    <row r="18" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="2" t="s">
+    <row r="18" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="102" t="s">
         <v>49</v>
       </c>
-      <c r="B18" s="29">
+      <c r="B18" s="110">
         <v>0.05</v>
       </c>
-      <c r="C18" s="35">
+      <c r="C18" s="109">
         <v>0.05</v>
       </c>
-      <c r="D18" s="35">
+      <c r="D18" s="109">
         <v>0.05</v>
       </c>
-      <c r="E18" s="30">
+      <c r="E18" s="120">
         <v>7.3999999999999996E-2</v>
       </c>
-      <c r="F18" s="101"/>
-      <c r="G18" s="25" t="s">
+      <c r="F18" s="96"/>
+      <c r="G18" s="24" t="s">
         <v>392</v>
       </c>
       <c r="H18" s="8" t="s">
         <v>463</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" s="2" t="s">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A19" s="102" t="s">
         <v>53</v>
       </c>
-      <c r="B19" s="20">
+      <c r="B19" s="107">
         <v>0.1</v>
       </c>
-      <c r="C19" s="32">
+      <c r="C19" s="109">
         <v>0.6</v>
       </c>
-      <c r="D19" s="32">
+      <c r="D19" s="109">
         <v>0.6</v>
       </c>
       <c r="E19" s="17"/>
-      <c r="F19" s="100"/>
+      <c r="F19" s="95"/>
       <c r="G19" s="18" t="s">
         <v>392</v>
       </c>
     </row>
-    <row r="20" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="2" t="s">
+    <row r="20" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="102" t="s">
         <v>54</v>
       </c>
-      <c r="B20" s="31">
+      <c r="B20" s="107">
         <v>0.03</v>
       </c>
-      <c r="C20" s="35">
+      <c r="C20" s="109">
         <v>0.6</v>
       </c>
-      <c r="D20" s="35">
+      <c r="D20" s="109">
         <v>0.6</v>
       </c>
-      <c r="E20" s="30"/>
-      <c r="F20" s="103"/>
-      <c r="G20" s="28"/>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A21" s="2" t="s">
+      <c r="E20" s="29"/>
+      <c r="F20" s="98"/>
+      <c r="G20" s="27"/>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A21" s="102" t="s">
         <v>57</v>
       </c>
-      <c r="B21" s="20">
+      <c r="B21" s="107">
         <v>0.15</v>
       </c>
-      <c r="C21" s="32">
+      <c r="C21" s="109">
         <v>0.7</v>
       </c>
-      <c r="D21" s="32">
+      <c r="D21" s="109">
         <v>0.7</v>
       </c>
       <c r="E21" s="17"/>
-      <c r="F21" s="100"/>
+      <c r="F21" s="95"/>
       <c r="G21" s="18" t="s">
         <v>392</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A22" s="2" t="s">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A22" s="102" t="s">
         <v>377</v>
       </c>
-      <c r="B22" s="36">
+      <c r="B22" s="122">
         <v>7.4999999999999997E-2</v>
       </c>
-      <c r="C22" s="32">
+      <c r="C22" s="109">
         <v>0.6</v>
       </c>
-      <c r="D22" s="32">
+      <c r="D22" s="109">
         <v>0.6</v>
       </c>
       <c r="E22" s="17"/>
-      <c r="F22" s="100"/>
+      <c r="F22" s="95"/>
       <c r="G22" s="19"/>
     </row>
-    <row r="23" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="2" t="s">
+    <row r="23" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="102" t="s">
         <v>62</v>
       </c>
-      <c r="B23" s="31">
+      <c r="B23" s="107">
         <v>0.02</v>
       </c>
-      <c r="C23" s="35">
+      <c r="C23" s="109">
         <v>0.6</v>
       </c>
-      <c r="D23" s="35">
+      <c r="D23" s="109">
         <v>0.4</v>
       </c>
-      <c r="E23" s="27"/>
-      <c r="F23" s="101"/>
-      <c r="G23" s="28"/>
-    </row>
-    <row r="24" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="2" t="s">
+      <c r="E23" s="26"/>
+      <c r="F23" s="96"/>
+      <c r="G23" s="27"/>
+    </row>
+    <row r="24" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="102" t="s">
         <v>378</v>
       </c>
-      <c r="B24" s="31">
+      <c r="B24" s="107">
         <v>0.1</v>
       </c>
-      <c r="C24" s="35">
+      <c r="C24" s="109">
         <v>0.6</v>
       </c>
-      <c r="D24" s="35">
+      <c r="D24" s="109">
         <v>0.6</v>
       </c>
-      <c r="E24" s="27"/>
-      <c r="F24" s="101"/>
-      <c r="G24" s="28"/>
-    </row>
-    <row r="25" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="2" t="s">
+      <c r="E24" s="26"/>
+      <c r="F24" s="96"/>
+      <c r="G24" s="27"/>
+    </row>
+    <row r="25" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="102" t="s">
         <v>63</v>
       </c>
-      <c r="B25" s="29">
+      <c r="B25" s="110">
         <v>0.1</v>
       </c>
-      <c r="C25" s="35">
+      <c r="C25" s="109">
         <v>0.6</v>
       </c>
-      <c r="D25" s="35">
+      <c r="D25" s="109">
         <v>0.6</v>
       </c>
-      <c r="E25" s="27"/>
-      <c r="F25" s="101"/>
-      <c r="G25" s="25" t="s">
+      <c r="E25" s="115"/>
+      <c r="F25" s="116"/>
+      <c r="G25" s="114" t="s">
         <v>387</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A26" s="2" t="s">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A26" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="B26" s="21">
+      <c r="B26" s="110">
         <v>0.1</v>
       </c>
-      <c r="C26" s="32"/>
-      <c r="D26" s="32">
+      <c r="C26" s="109"/>
+      <c r="D26" s="109">
         <v>1</v>
       </c>
       <c r="E26" s="16"/>
-      <c r="F26" s="97">
+      <c r="F26" s="92">
         <v>1</v>
       </c>
       <c r="G26" s="19"/>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A27" s="2" t="s">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A27" s="102" t="s">
         <v>65</v>
       </c>
-      <c r="B27" s="21">
+      <c r="B27" s="110">
         <v>0.1</v>
       </c>
-      <c r="C27" s="32"/>
-      <c r="D27" s="32">
+      <c r="C27" s="109"/>
+      <c r="D27" s="109">
         <v>1</v>
       </c>
       <c r="E27" s="16"/>
-      <c r="F27" s="97">
+      <c r="F27" s="92">
         <v>1</v>
       </c>
       <c r="G27" s="19"/>
     </row>
-    <row r="28" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="2" t="s">
+    <row r="28" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="102" t="s">
         <v>66</v>
       </c>
-      <c r="B28" s="31">
+      <c r="B28" s="107">
         <v>0.1</v>
       </c>
-      <c r="C28" s="24"/>
-      <c r="D28" s="35">
+      <c r="C28" s="111"/>
+      <c r="D28" s="109">
         <v>0.6</v>
       </c>
       <c r="E28" s="2"/>
-      <c r="F28" s="99"/>
-      <c r="G28" s="25" t="s">
+      <c r="F28" s="94"/>
+      <c r="G28" s="24" t="s">
         <v>387</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A29" s="2" t="s">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A29" s="102" t="s">
         <v>70</v>
       </c>
-      <c r="B29" s="20">
+      <c r="B29" s="107">
         <v>0.05</v>
       </c>
-      <c r="C29" s="32">
+      <c r="C29" s="109">
         <v>0.6</v>
       </c>
-      <c r="D29" s="32">
+      <c r="D29" s="109">
         <v>0.6</v>
       </c>
       <c r="E29" s="17"/>
-      <c r="F29" s="100"/>
+      <c r="F29" s="95"/>
       <c r="G29" s="18" t="s">
         <v>389</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A30" s="2" t="s">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A30" s="102" t="s">
         <v>71</v>
       </c>
-      <c r="B30" s="21">
+      <c r="B30" s="110">
         <v>0.05</v>
       </c>
-      <c r="C30" s="32">
+      <c r="C30" s="109">
         <v>1</v>
       </c>
-      <c r="D30" s="32">
+      <c r="D30" s="109">
         <v>1</v>
       </c>
       <c r="E30" s="17"/>
-      <c r="F30" s="100"/>
+      <c r="F30" s="95"/>
       <c r="G30" s="19"/>
     </row>
-    <row r="31" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="B31" s="29" t="s">
+      <c r="B31" s="28" t="s">
         <v>379</v>
       </c>
-      <c r="C31" s="34"/>
-      <c r="D31" s="34"/>
-      <c r="E31" s="27"/>
-      <c r="F31" s="101"/>
-      <c r="G31" s="25" t="s">
+      <c r="C31" s="32"/>
+      <c r="D31" s="32"/>
+      <c r="E31" s="26"/>
+      <c r="F31" s="96"/>
+      <c r="G31" s="24" t="s">
         <v>387</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A32" s="11" t="s">
         <v>83</v>
       </c>
-      <c r="B32" s="22">
+      <c r="B32" s="21">
         <v>20</v>
       </c>
-      <c r="C32" s="32"/>
-      <c r="D32" s="32">
+      <c r="C32" s="31"/>
+      <c r="D32" s="31">
         <v>1</v>
       </c>
       <c r="E32" s="17"/>
-      <c r="F32" s="100"/>
+      <c r="F32" s="95"/>
       <c r="G32" s="19"/>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A33" s="11" t="s">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A33" s="102" t="s">
         <v>84</v>
       </c>
-      <c r="B33" s="21" t="s">
+      <c r="B33" s="110" t="s">
         <v>380</v>
       </c>
-      <c r="C33" s="32">
+      <c r="C33" s="109">
         <v>3.95E-2</v>
       </c>
-      <c r="D33" s="32">
+      <c r="D33" s="109">
         <v>3.95E-2</v>
       </c>
-      <c r="E33" s="16"/>
-      <c r="F33" s="97">
+      <c r="E33" s="120"/>
+      <c r="F33" s="121">
         <v>3.95E-2</v>
       </c>
       <c r="G33" s="19"/>
@@ -3014,39 +3096,39 @@
         <v>463</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A34" s="11" t="s">
         <v>87</v>
       </c>
-      <c r="B34" s="21">
+      <c r="B34" s="20">
         <v>0.05</v>
       </c>
       <c r="C34" s="13"/>
       <c r="D34" s="14"/>
       <c r="E34" s="11"/>
-      <c r="F34" s="98"/>
+      <c r="F34" s="93"/>
       <c r="G34" s="18" t="s">
         <v>388</v>
       </c>
     </row>
-    <row r="35" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="2" t="s">
+    <row r="35" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="102" t="s">
         <v>462</v>
       </c>
-      <c r="B35" s="29">
+      <c r="B35" s="110">
         <v>0.05</v>
       </c>
-      <c r="C35" s="35"/>
-      <c r="D35" s="35">
+      <c r="C35" s="109"/>
+      <c r="D35" s="109">
         <v>3.5000000000000003E-2</v>
       </c>
-      <c r="E35" s="30">
+      <c r="E35" s="120">
         <v>3.5000000000000003E-2</v>
       </c>
-      <c r="F35" s="103">
+      <c r="F35" s="121">
         <v>3.5000000000000003E-2</v>
       </c>
-      <c r="G35" s="25" t="s">
+      <c r="G35" s="24" t="s">
         <v>387</v>
       </c>
     </row>
@@ -3064,23 +3146,23 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:K89"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="61.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.28515625" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="46.28515625" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="34.28515625" style="3" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="29.7109375" style="3" customWidth="1"/>
-    <col min="7" max="7" width="28.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="61.5546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.33203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="46.33203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="34.33203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="29.6640625" style="3" customWidth="1"/>
+    <col min="7" max="7" width="28.5546875" style="3" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="43" style="3" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="25.28515625" style="3" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.140625" style="3"/>
-    <col min="12" max="16384" width="9.140625" style="1"/>
+    <col min="9" max="9" width="18.88671875" style="3" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="25.33203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.109375" style="3"/>
+    <col min="12" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>91</v>
       </c>
@@ -3115,7 +3197,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="2" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2">
         <v>55</v>
       </c>
@@ -3140,7 +3222,7 @@
       <c r="J2" s="2"/>
       <c r="K2" s="2"/>
     </row>
-    <row r="3" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
         <v>34</v>
       </c>
@@ -3165,7 +3247,7 @@
       <c r="J3" s="2"/>
       <c r="K3" s="2"/>
     </row>
-    <row r="4" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
         <v>28</v>
       </c>
@@ -3188,7 +3270,7 @@
       <c r="J4" s="2"/>
       <c r="K4" s="2"/>
     </row>
-    <row r="5" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
         <v>6</v>
       </c>
@@ -3213,7 +3295,7 @@
       <c r="J5" s="2"/>
       <c r="K5" s="2"/>
     </row>
-    <row r="6" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
         <v>39</v>
       </c>
@@ -3236,7 +3318,7 @@
       <c r="J6" s="2"/>
       <c r="K6" s="2"/>
     </row>
-    <row r="7" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
         <v>58</v>
       </c>
@@ -3261,7 +3343,7 @@
       <c r="J7" s="2"/>
       <c r="K7" s="2"/>
     </row>
-    <row r="8" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
         <v>1</v>
       </c>
@@ -3288,7 +3370,7 @@
       <c r="J8" s="2"/>
       <c r="K8" s="2"/>
     </row>
-    <row r="9" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2">
         <v>29</v>
       </c>
@@ -3313,7 +3395,7 @@
       <c r="J9" s="2"/>
       <c r="K9" s="2"/>
     </row>
-    <row r="10" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2">
         <v>48</v>
       </c>
@@ -3340,7 +3422,7 @@
       <c r="J10" s="2"/>
       <c r="K10" s="2"/>
     </row>
-    <row r="11" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
         <v>18</v>
       </c>
@@ -3363,7 +3445,7 @@
       <c r="J11" s="2"/>
       <c r="K11" s="2"/>
     </row>
-    <row r="12" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2">
         <v>70</v>
       </c>
@@ -3386,7 +3468,7 @@
       <c r="J12" s="2"/>
       <c r="K12" s="2"/>
     </row>
-    <row r="13" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2">
         <v>60</v>
       </c>
@@ -3409,7 +3491,7 @@
       <c r="J13" s="2"/>
       <c r="K13" s="2"/>
     </row>
-    <row r="14" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2">
         <v>52</v>
       </c>
@@ -3436,7 +3518,7 @@
       <c r="J14" s="2"/>
       <c r="K14" s="2"/>
     </row>
-    <row r="15" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2">
         <v>47</v>
       </c>
@@ -3463,7 +3545,7 @@
       <c r="J15" s="2"/>
       <c r="K15" s="2"/>
     </row>
-    <row r="16" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2">
         <v>67</v>
       </c>
@@ -3490,7 +3572,7 @@
       <c r="J16" s="2"/>
       <c r="K16" s="2"/>
     </row>
-    <row r="17" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A17" s="2">
         <v>40</v>
       </c>
@@ -3513,7 +3595,7 @@
       <c r="J17" s="2"/>
       <c r="K17" s="2"/>
     </row>
-    <row r="18" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2">
         <v>53</v>
       </c>
@@ -3538,7 +3620,7 @@
       <c r="J18" s="2"/>
       <c r="K18" s="2"/>
     </row>
-    <row r="19" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A19" s="2">
         <v>22</v>
       </c>
@@ -3563,7 +3645,7 @@
       <c r="J19" s="2"/>
       <c r="K19" s="2"/>
     </row>
-    <row r="20" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A20" s="2">
         <v>84</v>
       </c>
@@ -3588,7 +3670,7 @@
       <c r="J20" s="2"/>
       <c r="K20" s="2"/>
     </row>
-    <row r="21" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A21" s="2">
         <v>9</v>
       </c>
@@ -3613,7 +3695,7 @@
       <c r="J21" s="2"/>
       <c r="K21" s="2"/>
     </row>
-    <row r="22" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A22" s="2">
         <v>30</v>
       </c>
@@ -3640,7 +3722,7 @@
       <c r="J22" s="2"/>
       <c r="K22" s="2"/>
     </row>
-    <row r="23" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A23" s="2">
         <v>75</v>
       </c>
@@ -3665,7 +3747,7 @@
       <c r="J23" s="2"/>
       <c r="K23" s="2"/>
     </row>
-    <row r="24" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A24" s="2">
         <v>59</v>
       </c>
@@ -3690,7 +3772,7 @@
       <c r="J24" s="2"/>
       <c r="K24" s="2"/>
     </row>
-    <row r="25" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A25" s="2">
         <v>31</v>
       </c>
@@ -3715,7 +3797,7 @@
       <c r="J25" s="2"/>
       <c r="K25" s="2"/>
     </row>
-    <row r="26" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A26" s="2">
         <v>62</v>
       </c>
@@ -3740,7 +3822,7 @@
       <c r="J26" s="2"/>
       <c r="K26" s="2"/>
     </row>
-    <row r="27" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A27" s="2">
         <v>41</v>
       </c>
@@ -3765,7 +3847,7 @@
       <c r="J27" s="2"/>
       <c r="K27" s="2"/>
     </row>
-    <row r="28" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A28" s="2">
         <v>63</v>
       </c>
@@ -3788,7 +3870,7 @@
       <c r="J28" s="2"/>
       <c r="K28" s="2"/>
     </row>
-    <row r="29" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A29" s="2">
         <v>71</v>
       </c>
@@ -3813,7 +3895,7 @@
       <c r="J29" s="2"/>
       <c r="K29" s="2"/>
     </row>
-    <row r="30" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A30" s="2">
         <v>69</v>
       </c>
@@ -3840,7 +3922,7 @@
       <c r="J30" s="2"/>
       <c r="K30" s="2"/>
     </row>
-    <row r="31" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" s="8" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A31" s="7">
         <v>27</v>
       </c>
@@ -3859,7 +3941,7 @@
       <c r="J31" s="7"/>
       <c r="K31" s="7"/>
     </row>
-    <row r="32" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A32" s="2">
         <v>78</v>
       </c>
@@ -3882,7 +3964,7 @@
       <c r="J32" s="2"/>
       <c r="K32" s="2"/>
     </row>
-    <row r="33" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A33" s="2">
         <v>80</v>
       </c>
@@ -3909,7 +3991,7 @@
       <c r="J33" s="2"/>
       <c r="K33" s="2"/>
     </row>
-    <row r="34" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A34" s="2">
         <v>86</v>
       </c>
@@ -3936,7 +4018,7 @@
       <c r="J34" s="2"/>
       <c r="K34" s="2"/>
     </row>
-    <row r="35" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A35" s="2">
         <v>19</v>
       </c>
@@ -3963,7 +4045,7 @@
       <c r="J35" s="2"/>
       <c r="K35" s="2"/>
     </row>
-    <row r="36" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A36" s="2">
         <v>81</v>
       </c>
@@ -3990,7 +4072,7 @@
       <c r="J36" s="2"/>
       <c r="K36" s="2"/>
     </row>
-    <row r="37" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A37" s="2">
         <v>82</v>
       </c>
@@ -4009,7 +4091,7 @@
       <c r="J37" s="2"/>
       <c r="K37" s="2"/>
     </row>
-    <row r="38" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A38" s="2">
         <v>36</v>
       </c>
@@ -4034,7 +4116,7 @@
       <c r="J38" s="2"/>
       <c r="K38" s="2"/>
     </row>
-    <row r="39" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A39" s="2">
         <v>88</v>
       </c>
@@ -4061,7 +4143,7 @@
       <c r="J39" s="2"/>
       <c r="K39" s="2"/>
     </row>
-    <row r="40" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A40" s="2">
         <v>12</v>
       </c>
@@ -4088,7 +4170,7 @@
       <c r="J40" s="2"/>
       <c r="K40" s="2"/>
     </row>
-    <row r="41" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A41" s="2">
         <v>26</v>
       </c>
@@ -4115,7 +4197,7 @@
       <c r="J41" s="2"/>
       <c r="K41" s="2"/>
     </row>
-    <row r="42" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A42" s="2">
         <v>17</v>
       </c>
@@ -4142,7 +4224,7 @@
       <c r="J42" s="2"/>
       <c r="K42" s="2"/>
     </row>
-    <row r="43" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A43" s="2">
         <v>20</v>
       </c>
@@ -4173,7 +4255,7 @@
       </c>
       <c r="K43" s="2"/>
     </row>
-    <row r="44" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A44" s="2">
         <v>38</v>
       </c>
@@ -4198,7 +4280,7 @@
       <c r="J44" s="2"/>
       <c r="K44" s="2"/>
     </row>
-    <row r="45" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A45" s="2">
         <v>50</v>
       </c>
@@ -4221,7 +4303,7 @@
       <c r="J45" s="2"/>
       <c r="K45" s="2"/>
     </row>
-    <row r="46" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A46" s="2">
         <v>76</v>
       </c>
@@ -4248,7 +4330,7 @@
       <c r="J46" s="2"/>
       <c r="K46" s="2"/>
     </row>
-    <row r="47" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A47" s="2">
         <v>25</v>
       </c>
@@ -4273,7 +4355,7 @@
       <c r="J47" s="2"/>
       <c r="K47" s="2"/>
     </row>
-    <row r="48" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A48" s="2">
         <v>61</v>
       </c>
@@ -4296,7 +4378,7 @@
       <c r="J48" s="2"/>
       <c r="K48" s="2"/>
     </row>
-    <row r="49" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A49" s="2">
         <v>13</v>
       </c>
@@ -4321,7 +4403,7 @@
       <c r="J49" s="2"/>
       <c r="K49" s="2"/>
     </row>
-    <row r="50" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A50" s="2">
         <v>7</v>
       </c>
@@ -4344,7 +4426,7 @@
       <c r="J50" s="2"/>
       <c r="K50" s="2"/>
     </row>
-    <row r="51" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A51" s="2">
         <v>87</v>
       </c>
@@ -4371,7 +4453,7 @@
       <c r="J51" s="2"/>
       <c r="K51" s="2"/>
     </row>
-    <row r="52" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A52" s="2">
         <v>64</v>
       </c>
@@ -4398,7 +4480,7 @@
       <c r="J52" s="2"/>
       <c r="K52" s="2"/>
     </row>
-    <row r="53" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A53" s="2">
         <v>45</v>
       </c>
@@ -4423,7 +4505,7 @@
       <c r="J53" s="2"/>
       <c r="K53" s="2"/>
     </row>
-    <row r="54" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A54" s="2">
         <v>11</v>
       </c>
@@ -4450,7 +4532,7 @@
       <c r="J54" s="2"/>
       <c r="K54" s="2"/>
     </row>
-    <row r="55" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A55" s="2">
         <v>32</v>
       </c>
@@ -4475,7 +4557,7 @@
       <c r="J55" s="2"/>
       <c r="K55" s="2"/>
     </row>
-    <row r="56" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A56" s="2">
         <v>24</v>
       </c>
@@ -4502,7 +4584,7 @@
       <c r="J56" s="2"/>
       <c r="K56" s="2"/>
     </row>
-    <row r="57" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A57" s="2">
         <v>4</v>
       </c>
@@ -4527,7 +4609,7 @@
       <c r="J57" s="2"/>
       <c r="K57" s="2"/>
     </row>
-    <row r="58" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A58" s="2">
         <v>56</v>
       </c>
@@ -4552,7 +4634,7 @@
       <c r="J58" s="2"/>
       <c r="K58" s="2"/>
     </row>
-    <row r="59" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A59" s="2">
         <v>66</v>
       </c>
@@ -4579,7 +4661,7 @@
       <c r="J59" s="2"/>
       <c r="K59" s="2"/>
     </row>
-    <row r="60" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A60" s="2">
         <v>79</v>
       </c>
@@ -4604,7 +4686,7 @@
       <c r="J60" s="2"/>
       <c r="K60" s="2"/>
     </row>
-    <row r="61" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A61" s="2">
         <v>33</v>
       </c>
@@ -4629,7 +4711,7 @@
       <c r="J61" s="2"/>
       <c r="K61" s="2"/>
     </row>
-    <row r="62" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A62" s="2">
         <v>3</v>
       </c>
@@ -4654,7 +4736,7 @@
       <c r="J62" s="2"/>
       <c r="K62" s="2"/>
     </row>
-    <row r="63" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A63" s="2">
         <v>46</v>
       </c>
@@ -4677,7 +4759,7 @@
       <c r="J63" s="2"/>
       <c r="K63" s="2"/>
     </row>
-    <row r="64" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A64" s="2">
         <v>44</v>
       </c>
@@ -4702,7 +4784,7 @@
       <c r="J64" s="2"/>
       <c r="K64" s="2"/>
     </row>
-    <row r="65" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A65" s="2">
         <v>14</v>
       </c>
@@ -4727,7 +4809,7 @@
       <c r="J65" s="2"/>
       <c r="K65" s="2"/>
     </row>
-    <row r="66" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A66" s="2">
         <v>83</v>
       </c>
@@ -4754,7 +4836,7 @@
       <c r="J66" s="2"/>
       <c r="K66" s="2"/>
     </row>
-    <row r="67" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A67" s="2">
         <v>16</v>
       </c>
@@ -4781,7 +4863,7 @@
       <c r="J67" s="2"/>
       <c r="K67" s="2"/>
     </row>
-    <row r="68" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A68" s="2">
         <v>35</v>
       </c>
@@ -4808,7 +4890,7 @@
       <c r="J68" s="2"/>
       <c r="K68" s="2"/>
     </row>
-    <row r="69" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A69" s="2">
         <v>68</v>
       </c>
@@ -4837,7 +4919,7 @@
       <c r="J69" s="2"/>
       <c r="K69" s="2"/>
     </row>
-    <row r="70" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A70" s="2">
         <v>10</v>
       </c>
@@ -4862,7 +4944,7 @@
       <c r="J70" s="2"/>
       <c r="K70" s="2"/>
     </row>
-    <row r="71" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A71" s="2">
         <v>2</v>
       </c>
@@ -4887,7 +4969,7 @@
       <c r="J71" s="2"/>
       <c r="K71" s="2"/>
     </row>
-    <row r="72" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A72" s="2">
         <v>85</v>
       </c>
@@ -4914,7 +4996,7 @@
       <c r="J72" s="2"/>
       <c r="K72" s="2"/>
     </row>
-    <row r="73" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A73" s="2">
         <v>21</v>
       </c>
@@ -4941,7 +5023,7 @@
       <c r="J73" s="2"/>
       <c r="K73" s="2"/>
     </row>
-    <row r="74" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A74" s="2">
         <v>57</v>
       </c>
@@ -4968,7 +5050,7 @@
       <c r="J74" s="2"/>
       <c r="K74" s="2"/>
     </row>
-    <row r="75" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A75" s="2">
         <v>72</v>
       </c>
@@ -4995,7 +5077,7 @@
       <c r="J75" s="2"/>
       <c r="K75" s="2"/>
     </row>
-    <row r="76" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A76" s="2">
         <v>65</v>
       </c>
@@ -5018,7 +5100,7 @@
       <c r="J76" s="2"/>
       <c r="K76" s="2"/>
     </row>
-    <row r="77" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A77" s="2">
         <v>43</v>
       </c>
@@ -5043,7 +5125,7 @@
       <c r="J77" s="2"/>
       <c r="K77" s="2"/>
     </row>
-    <row r="78" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A78" s="2">
         <v>74</v>
       </c>
@@ -5066,7 +5148,7 @@
       <c r="J78" s="2"/>
       <c r="K78" s="2"/>
     </row>
-    <row r="79" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A79" s="2">
         <v>54</v>
       </c>
@@ -5093,7 +5175,7 @@
       <c r="J79" s="2"/>
       <c r="K79" s="2"/>
     </row>
-    <row r="80" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A80" s="2">
         <v>49</v>
       </c>
@@ -5120,7 +5202,7 @@
       <c r="J80" s="2"/>
       <c r="K80" s="2"/>
     </row>
-    <row r="81" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A81" s="2">
         <v>37</v>
       </c>
@@ -5145,7 +5227,7 @@
       <c r="J81" s="2"/>
       <c r="K81" s="2"/>
     </row>
-    <row r="82" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A82" s="2">
         <v>42</v>
       </c>
@@ -5172,7 +5254,7 @@
       <c r="J82" s="2"/>
       <c r="K82" s="2"/>
     </row>
-    <row r="83" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A83" s="2">
         <v>23</v>
       </c>
@@ -5199,7 +5281,7 @@
       <c r="J83" s="2"/>
       <c r="K83" s="2"/>
     </row>
-    <row r="84" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A84" s="2">
         <v>8</v>
       </c>
@@ -5226,7 +5308,7 @@
       <c r="J84" s="2"/>
       <c r="K84" s="2"/>
     </row>
-    <row r="85" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A85" s="2">
         <v>51</v>
       </c>
@@ -5245,7 +5327,7 @@
       <c r="J85" s="2"/>
       <c r="K85" s="2"/>
     </row>
-    <row r="86" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A86" s="2">
         <v>15</v>
       </c>
@@ -5272,7 +5354,7 @@
       <c r="J86" s="2"/>
       <c r="K86" s="2"/>
     </row>
-    <row r="87" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A87" s="2">
         <v>73</v>
       </c>
@@ -5297,7 +5379,7 @@
       <c r="J87" s="2"/>
       <c r="K87" s="2"/>
     </row>
-    <row r="88" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A88" s="2">
         <v>77</v>
       </c>
@@ -5324,7 +5406,7 @@
       <c r="J88" s="2"/>
       <c r="K88" s="2"/>
     </row>
-    <row r="89" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A89" s="2">
         <v>5</v>
       </c>
@@ -5369,840 +5451,840 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B76C84A3-BB4C-4959-9F37-D2E2982D3050}">
   <dimension ref="A1:H45"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="61.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="95.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="95.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="61.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="95.5546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="95.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="105" t="s">
+    <row r="1" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="99" t="s">
         <v>393</v>
       </c>
-      <c r="B1" s="106"/>
-      <c r="C1" s="106"/>
-      <c r="D1" s="106"/>
-      <c r="E1" s="106"/>
-      <c r="F1" s="107"/>
-    </row>
-    <row r="2" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="41" t="s">
+      <c r="B1" s="100"/>
+      <c r="C1" s="100"/>
+      <c r="D1" s="100"/>
+      <c r="E1" s="100"/>
+      <c r="F1" s="101"/>
+    </row>
+    <row r="2" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="36" t="s">
         <v>394</v>
       </c>
-      <c r="B2" s="42" t="s">
+      <c r="B2" s="37" t="s">
         <v>395</v>
       </c>
-      <c r="C2" s="42" t="s">
+      <c r="C2" s="37" t="s">
         <v>396</v>
       </c>
-      <c r="D2" s="42" t="s">
+      <c r="D2" s="37" t="s">
         <v>397</v>
       </c>
-      <c r="E2" s="42" t="s">
+      <c r="E2" s="37" t="s">
         <v>398</v>
       </c>
-      <c r="F2" s="43" t="s">
+      <c r="F2" s="38" t="s">
         <v>399</v>
       </c>
-      <c r="G2" s="44" t="s">
+      <c r="G2" s="39" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="45" t="s">
+    <row r="3" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="40" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="46"/>
-      <c r="C3" s="46">
+      <c r="B3" s="41"/>
+      <c r="C3" s="41">
         <v>1.4999999999999999E-2</v>
       </c>
-      <c r="D3" s="46">
+      <c r="D3" s="41">
         <v>1.4999999999999999E-2</v>
       </c>
-      <c r="E3" s="46">
+      <c r="E3" s="41">
         <v>1.4999999999999999E-2</v>
       </c>
-      <c r="F3" s="47">
+      <c r="F3" s="42">
         <v>0.2</v>
       </c>
-      <c r="G3" s="48"/>
-    </row>
-    <row r="4" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="45" t="s">
+      <c r="G3" s="43"/>
+    </row>
+    <row r="4" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="40" t="s">
         <v>400</v>
       </c>
-      <c r="B4" s="46">
+      <c r="B4" s="41">
         <v>0.01</v>
       </c>
-      <c r="C4" s="46">
+      <c r="C4" s="41">
         <v>0.01</v>
       </c>
-      <c r="D4" s="46"/>
-      <c r="E4" s="46"/>
-      <c r="F4" s="47">
+      <c r="D4" s="41"/>
+      <c r="E4" s="41"/>
+      <c r="F4" s="42">
         <v>6.5000000000000002E-2</v>
       </c>
-      <c r="G4" s="48"/>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="49" t="s">
+      <c r="G4" s="43"/>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" s="44" t="s">
         <v>401</v>
       </c>
-      <c r="B5" s="50">
+      <c r="B5" s="45">
         <v>0.01</v>
       </c>
-      <c r="C5" s="50">
+      <c r="C5" s="45">
         <v>0.01</v>
       </c>
-      <c r="D5" s="50"/>
-      <c r="E5" s="50"/>
-      <c r="F5" s="50">
+      <c r="D5" s="45"/>
+      <c r="E5" s="45"/>
+      <c r="F5" s="45">
         <v>6.5000000000000002E-2</v>
       </c>
-      <c r="G5" s="51" t="s">
+      <c r="G5" s="46" t="s">
         <v>402</v>
       </c>
-      <c r="H5" s="52"/>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" s="53" t="s">
+      <c r="H5" s="47"/>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" s="48" t="s">
         <v>403</v>
       </c>
-      <c r="B6" s="54"/>
-      <c r="C6" s="54">
+      <c r="B6" s="49"/>
+      <c r="C6" s="49">
         <v>1</v>
       </c>
-      <c r="D6" s="54"/>
-      <c r="E6" s="54">
+      <c r="D6" s="49"/>
+      <c r="E6" s="49">
         <v>1</v>
       </c>
-      <c r="F6" s="54">
+      <c r="F6" s="49">
         <v>0.2</v>
       </c>
-      <c r="G6" s="55" t="s">
+      <c r="G6" s="50" t="s">
         <v>404</v>
       </c>
-      <c r="H6" s="56"/>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" s="57" t="s">
+      <c r="H6" s="51"/>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" s="52" t="s">
         <v>405</v>
       </c>
-      <c r="B7" s="58"/>
-      <c r="C7" s="58">
+      <c r="B7" s="53"/>
+      <c r="C7" s="53">
         <v>1.4999999999999999E-2</v>
       </c>
-      <c r="D7" s="58"/>
-      <c r="E7" s="58">
+      <c r="D7" s="53"/>
+      <c r="E7" s="53">
         <v>1.4999999999999999E-2</v>
       </c>
-      <c r="F7" s="58"/>
-      <c r="G7" s="59"/>
-      <c r="H7" s="52"/>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" s="57" t="s">
+      <c r="F7" s="53"/>
+      <c r="G7" s="54"/>
+      <c r="H7" s="47"/>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8" s="52" t="s">
         <v>406</v>
       </c>
-      <c r="B8" s="58"/>
-      <c r="C8" s="58"/>
-      <c r="D8" s="58"/>
-      <c r="E8" s="58"/>
-      <c r="F8" s="58">
+      <c r="B8" s="53"/>
+      <c r="C8" s="53"/>
+      <c r="D8" s="53"/>
+      <c r="E8" s="53"/>
+      <c r="F8" s="53">
         <v>6.5000000000000002E-2</v>
       </c>
-      <c r="G8" s="60" t="s">
+      <c r="G8" s="55" t="s">
         <v>407</v>
       </c>
-      <c r="H8" s="56" t="s">
+      <c r="H8" s="51" t="s">
         <v>408</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" s="57" t="s">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" s="52" t="s">
         <v>409</v>
       </c>
-      <c r="B9" s="58"/>
-      <c r="C9" s="58">
+      <c r="B9" s="53"/>
+      <c r="C9" s="53">
         <v>0.01</v>
       </c>
-      <c r="D9" s="58"/>
-      <c r="E9" s="58">
+      <c r="D9" s="53"/>
+      <c r="E9" s="53">
         <v>0.01</v>
       </c>
-      <c r="F9" s="58">
+      <c r="F9" s="53">
         <v>6.5000000000000002E-2</v>
       </c>
-      <c r="G9" s="59"/>
-      <c r="H9" s="52"/>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="57" t="s">
+      <c r="G9" s="54"/>
+      <c r="H9" s="47"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10" s="52" t="s">
         <v>410</v>
       </c>
-      <c r="B10" s="58">
+      <c r="B10" s="53">
         <v>0.01</v>
       </c>
-      <c r="C10" s="58">
+      <c r="C10" s="53">
         <v>0.01</v>
       </c>
-      <c r="D10" s="58"/>
-      <c r="E10" s="58"/>
-      <c r="F10" s="58">
+      <c r="D10" s="53"/>
+      <c r="E10" s="53"/>
+      <c r="F10" s="53">
         <v>6.5000000000000002E-2</v>
       </c>
-      <c r="G10" s="59" t="s">
+      <c r="G10" s="54" t="s">
         <v>411</v>
       </c>
-      <c r="H10" s="61"/>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" s="62" t="s">
+      <c r="H10" s="56"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A11" s="57" t="s">
         <v>412</v>
       </c>
-      <c r="B11" s="63"/>
-      <c r="C11" s="63">
+      <c r="B11" s="58"/>
+      <c r="C11" s="58">
         <v>0.01</v>
       </c>
-      <c r="D11" s="63"/>
-      <c r="E11" s="63"/>
-      <c r="F11" s="63">
+      <c r="D11" s="58"/>
+      <c r="E11" s="58"/>
+      <c r="F11" s="58">
         <v>0.2</v>
       </c>
-      <c r="G11" s="64"/>
-      <c r="H11" s="52"/>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" s="65" t="s">
+      <c r="G11" s="59"/>
+      <c r="H11" s="47"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A12" s="60" t="s">
         <v>413</v>
       </c>
-      <c r="B12" s="58"/>
-      <c r="C12" s="58"/>
-      <c r="D12" s="58"/>
-      <c r="E12" s="58"/>
-      <c r="F12" s="58">
+      <c r="B12" s="53"/>
+      <c r="C12" s="53"/>
+      <c r="D12" s="53"/>
+      <c r="E12" s="53"/>
+      <c r="F12" s="53">
         <v>6.5000000000000002E-2</v>
       </c>
-      <c r="G12" s="60"/>
-      <c r="H12" s="56" t="s">
+      <c r="G12" s="55"/>
+      <c r="H12" s="51" t="s">
         <v>408</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A13" s="57" t="s">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A13" s="52" t="s">
         <v>414</v>
       </c>
-      <c r="B13" s="58">
+      <c r="B13" s="53">
         <v>0.01</v>
       </c>
-      <c r="C13" s="58">
+      <c r="C13" s="53">
         <v>0.01</v>
       </c>
-      <c r="D13" s="58"/>
-      <c r="E13" s="58">
+      <c r="D13" s="53"/>
+      <c r="E13" s="53">
         <v>0.01</v>
       </c>
-      <c r="F13" s="58">
+      <c r="F13" s="53">
         <v>0.2</v>
       </c>
-      <c r="G13" s="66" t="s">
+      <c r="G13" s="61" t="s">
         <v>415</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14" s="57" t="s">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A14" s="52" t="s">
         <v>44</v>
       </c>
-      <c r="B14" s="58"/>
-      <c r="C14" s="58">
+      <c r="B14" s="53"/>
+      <c r="C14" s="53">
         <v>1.4999999999999999E-2</v>
       </c>
-      <c r="D14" s="58">
+      <c r="D14" s="53">
         <v>1.4999999999999999E-2</v>
       </c>
-      <c r="E14" s="58"/>
-      <c r="F14" s="58">
+      <c r="E14" s="53"/>
+      <c r="F14" s="53">
         <v>0</v>
       </c>
-      <c r="G14" s="59" t="s">
+      <c r="G14" s="54" t="s">
         <v>416</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" s="57" t="s">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A15" s="52" t="s">
         <v>417</v>
       </c>
-      <c r="B15" s="58"/>
-      <c r="C15" s="58"/>
-      <c r="D15" s="58"/>
-      <c r="E15" s="58"/>
-      <c r="F15" s="58">
+      <c r="B15" s="53"/>
+      <c r="C15" s="53"/>
+      <c r="D15" s="53"/>
+      <c r="E15" s="53"/>
+      <c r="F15" s="53">
         <v>6.5000000000000002E-2</v>
       </c>
-      <c r="G15" s="60" t="s">
+      <c r="G15" s="55" t="s">
         <v>418</v>
       </c>
-      <c r="H15" s="67" t="s">
+      <c r="H15" s="62" t="s">
         <v>419</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A16" s="68" t="s">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A16" s="63" t="s">
         <v>420</v>
       </c>
-      <c r="B16" s="69">
+      <c r="B16" s="64">
         <v>0.05</v>
       </c>
-      <c r="C16" s="69"/>
-      <c r="D16" s="69"/>
-      <c r="E16" s="69"/>
-      <c r="F16" s="69"/>
-      <c r="G16" s="70" t="s">
+      <c r="C16" s="64"/>
+      <c r="D16" s="64"/>
+      <c r="E16" s="64"/>
+      <c r="F16" s="64"/>
+      <c r="G16" s="65" t="s">
         <v>421</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17" s="68" t="s">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A17" s="63" t="s">
         <v>47</v>
       </c>
-      <c r="B17" s="69"/>
-      <c r="C17" s="69">
+      <c r="B17" s="64"/>
+      <c r="C17" s="64">
         <v>2.18E-2</v>
       </c>
-      <c r="D17" s="69"/>
-      <c r="E17" s="69">
+      <c r="D17" s="64"/>
+      <c r="E17" s="64">
         <v>2.18E-2</v>
       </c>
-      <c r="F17" s="69">
+      <c r="F17" s="64">
         <v>6.5000000000000002E-2</v>
       </c>
-      <c r="G17" s="71" t="s">
+      <c r="G17" s="66" t="s">
         <v>422</v>
       </c>
-      <c r="H17" s="67" t="s">
+      <c r="H17" s="62" t="s">
         <v>423</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A18" s="68" t="s">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A18" s="63" t="s">
         <v>424</v>
       </c>
-      <c r="B18" s="69"/>
-      <c r="C18" s="69"/>
-      <c r="D18" s="69"/>
-      <c r="E18" s="69"/>
-      <c r="F18" s="69"/>
-      <c r="G18" s="72" t="s">
+      <c r="B18" s="64"/>
+      <c r="C18" s="64"/>
+      <c r="D18" s="64"/>
+      <c r="E18" s="64"/>
+      <c r="F18" s="64"/>
+      <c r="G18" s="67" t="s">
         <v>425</v>
       </c>
-      <c r="H18" s="67" t="s">
+      <c r="H18" s="62" t="s">
         <v>426</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" s="73" t="s">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A19" s="68" t="s">
         <v>49</v>
       </c>
-      <c r="B19" s="74">
+      <c r="B19" s="69">
         <v>0.05</v>
       </c>
-      <c r="C19" s="74">
+      <c r="C19" s="69">
         <v>0.05</v>
       </c>
-      <c r="D19" s="74">
+      <c r="D19" s="69">
         <v>7.3999999999999996E-2</v>
       </c>
-      <c r="E19" s="74"/>
-      <c r="F19" s="74">
+      <c r="E19" s="69"/>
+      <c r="F19" s="69">
         <v>0</v>
       </c>
-      <c r="G19" s="75" t="s">
+      <c r="G19" s="70" t="s">
         <v>427</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" s="57" t="s">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A20" s="52" t="s">
         <v>50</v>
       </c>
-      <c r="B20" s="58">
+      <c r="B20" s="53">
         <v>1.4999999999999999E-2</v>
       </c>
-      <c r="C20" s="58">
+      <c r="C20" s="53">
         <v>1.4999999999999999E-2</v>
       </c>
-      <c r="D20" s="58"/>
-      <c r="E20" s="58">
+      <c r="D20" s="53"/>
+      <c r="E20" s="53">
         <v>1.4999999999999999E-2</v>
       </c>
-      <c r="F20" s="58">
+      <c r="F20" s="53">
         <v>0</v>
       </c>
-      <c r="G20" s="60"/>
-      <c r="H20" s="52"/>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A21" s="57" t="s">
+      <c r="G20" s="55"/>
+      <c r="H20" s="47"/>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A21" s="52" t="s">
         <v>428</v>
       </c>
-      <c r="B21" s="58">
+      <c r="B21" s="53">
         <v>0.01</v>
       </c>
-      <c r="C21" s="58">
+      <c r="C21" s="53">
         <v>0.01</v>
       </c>
-      <c r="D21" s="58"/>
-      <c r="E21" s="58"/>
-      <c r="F21" s="58">
+      <c r="D21" s="53"/>
+      <c r="E21" s="53"/>
+      <c r="F21" s="53">
         <v>6.5000000000000002E-2</v>
       </c>
-      <c r="G21" s="60"/>
-      <c r="H21" s="52"/>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A22" s="76" t="s">
+      <c r="G21" s="55"/>
+      <c r="H21" s="47"/>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A22" s="71" t="s">
         <v>54</v>
       </c>
-      <c r="B22" s="77"/>
-      <c r="C22" s="77">
+      <c r="B22" s="72"/>
+      <c r="C22" s="72">
         <v>1.4999999999999999E-2</v>
       </c>
-      <c r="D22" s="77"/>
-      <c r="E22" s="77">
+      <c r="D22" s="72"/>
+      <c r="E22" s="72">
         <v>1.4999999999999999E-2</v>
       </c>
-      <c r="F22" s="77">
+      <c r="F22" s="72">
         <v>0.2</v>
       </c>
-      <c r="G22" s="78" t="s">
+      <c r="G22" s="73" t="s">
         <v>429</v>
       </c>
-      <c r="H22" s="67" t="s">
+      <c r="H22" s="62" t="s">
         <v>430</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A23" s="57" t="s">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A23" s="52" t="s">
         <v>56</v>
       </c>
-      <c r="B23" s="58"/>
-      <c r="C23" s="58">
+      <c r="B23" s="53"/>
+      <c r="C23" s="53">
         <v>0.01</v>
       </c>
-      <c r="D23" s="58">
+      <c r="D23" s="53">
         <v>0.01</v>
       </c>
-      <c r="E23" s="58"/>
-      <c r="F23" s="58">
+      <c r="E23" s="53"/>
+      <c r="F23" s="53">
         <v>6.5000000000000002E-2</v>
       </c>
-      <c r="G23" s="79"/>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A24" s="57" t="s">
+      <c r="G23" s="74"/>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A24" s="52" t="s">
         <v>57</v>
       </c>
-      <c r="B24" s="58"/>
-      <c r="C24" s="58">
+      <c r="B24" s="53"/>
+      <c r="C24" s="53">
         <v>0.02</v>
       </c>
-      <c r="D24" s="58"/>
-      <c r="E24" s="58"/>
-      <c r="F24" s="58"/>
-      <c r="G24" s="60"/>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A25" s="57" t="s">
+      <c r="D24" s="53"/>
+      <c r="E24" s="53"/>
+      <c r="F24" s="53"/>
+      <c r="G24" s="55"/>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A25" s="52" t="s">
         <v>431</v>
       </c>
-      <c r="B25" s="58"/>
-      <c r="C25" s="58">
+      <c r="B25" s="53"/>
+      <c r="C25" s="53">
         <v>4.2000000000000003E-2</v>
       </c>
-      <c r="D25" s="58"/>
-      <c r="E25" s="58"/>
-      <c r="F25" s="58">
+      <c r="D25" s="53"/>
+      <c r="E25" s="53"/>
+      <c r="F25" s="53">
         <v>6.5000000000000002E-2</v>
       </c>
-      <c r="G25" s="60" t="s">
+      <c r="G25" s="55" t="s">
         <v>432</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A26" s="57" t="s">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A26" s="52" t="s">
         <v>433</v>
       </c>
-      <c r="B26" s="58">
+      <c r="B26" s="53">
         <v>0.01</v>
       </c>
-      <c r="C26" s="58">
+      <c r="C26" s="53">
         <v>0.01</v>
       </c>
-      <c r="D26" s="58"/>
-      <c r="E26" s="58"/>
-      <c r="F26" s="58">
+      <c r="D26" s="53"/>
+      <c r="E26" s="53"/>
+      <c r="F26" s="53">
         <v>0.2</v>
       </c>
-      <c r="G26" s="80"/>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A27" s="68" t="s">
+      <c r="G26" s="75"/>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A27" s="63" t="s">
         <v>434</v>
       </c>
-      <c r="B27" s="69">
+      <c r="B27" s="64">
         <v>0.01</v>
       </c>
-      <c r="C27" s="69">
+      <c r="C27" s="64">
         <v>0.01</v>
       </c>
-      <c r="D27" s="69"/>
-      <c r="E27" s="69"/>
-      <c r="F27" s="69">
+      <c r="D27" s="64"/>
+      <c r="E27" s="64"/>
+      <c r="F27" s="64">
         <v>0.2</v>
       </c>
-      <c r="G27" s="81" t="s">
+      <c r="G27" s="76" t="s">
         <v>435</v>
       </c>
-      <c r="H27" s="67" t="s">
+      <c r="H27" s="62" t="s">
         <v>436</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A28" s="68" t="s">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A28" s="63" t="s">
         <v>437</v>
       </c>
-      <c r="B28" s="69">
+      <c r="B28" s="64">
         <v>1.4999999999999999E-2</v>
       </c>
-      <c r="C28" s="69">
+      <c r="C28" s="64">
         <v>1.4999999999999999E-2</v>
       </c>
-      <c r="D28" s="69"/>
-      <c r="E28" s="69"/>
-      <c r="F28" s="69">
+      <c r="D28" s="64"/>
+      <c r="E28" s="64"/>
+      <c r="F28" s="64">
         <v>6.5000000000000002E-2</v>
       </c>
-      <c r="G28" s="82" t="s">
+      <c r="G28" s="77" t="s">
         <v>438</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A29" s="57" t="s">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A29" s="52" t="s">
         <v>439</v>
       </c>
-      <c r="B29" s="58">
+      <c r="B29" s="53">
         <v>1.4999999999999999E-2</v>
       </c>
-      <c r="C29" s="58">
+      <c r="C29" s="53">
         <v>1.4999999999999999E-2</v>
       </c>
-      <c r="D29" s="58"/>
-      <c r="E29" s="58"/>
-      <c r="F29" s="58">
+      <c r="D29" s="53"/>
+      <c r="E29" s="53"/>
+      <c r="F29" s="53">
         <v>6.5000000000000002E-2</v>
       </c>
-      <c r="G29" s="60" t="s">
+      <c r="G29" s="55" t="s">
         <v>387</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A30" s="57" t="s">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A30" s="52" t="s">
         <v>440</v>
       </c>
-      <c r="B30" s="58"/>
-      <c r="C30" s="58"/>
-      <c r="D30" s="58"/>
-      <c r="E30" s="58"/>
-      <c r="F30" s="58">
+      <c r="B30" s="53"/>
+      <c r="C30" s="53"/>
+      <c r="D30" s="53"/>
+      <c r="E30" s="53"/>
+      <c r="F30" s="53">
         <v>0.15</v>
       </c>
-      <c r="G30" s="60" t="s">
+      <c r="G30" s="55" t="s">
         <v>441</v>
       </c>
-      <c r="H30" s="67"/>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A31" s="83" t="s">
+      <c r="H30" s="62"/>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A31" s="78" t="s">
         <v>442</v>
       </c>
-      <c r="B31" s="84">
+      <c r="B31" s="79">
         <v>0.01</v>
       </c>
-      <c r="C31" s="84">
+      <c r="C31" s="79">
         <v>0.01</v>
       </c>
-      <c r="D31" s="84"/>
-      <c r="E31" s="84"/>
-      <c r="F31" s="84">
+      <c r="D31" s="79"/>
+      <c r="E31" s="79"/>
+      <c r="F31" s="79">
         <v>0.2</v>
       </c>
-      <c r="G31" s="85" t="s">
+      <c r="G31" s="80" t="s">
         <v>443</v>
       </c>
-      <c r="H31" s="67" t="s">
+      <c r="H31" s="62" t="s">
         <v>408</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A32" s="60" t="s">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A32" s="55" t="s">
         <v>444</v>
       </c>
-      <c r="B32" s="58"/>
-      <c r="C32" s="58"/>
-      <c r="D32" s="58"/>
-      <c r="E32" s="58"/>
-      <c r="F32" s="58">
+      <c r="B32" s="53"/>
+      <c r="C32" s="53"/>
+      <c r="D32" s="53"/>
+      <c r="E32" s="53"/>
+      <c r="F32" s="53">
         <v>6.5000000000000002E-2</v>
       </c>
-      <c r="G32" s="86" t="s">
+      <c r="G32" s="81" t="s">
         <v>445</v>
       </c>
-      <c r="H32" s="67"/>
-    </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A33" s="53" t="s">
+      <c r="H32" s="62"/>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A33" s="48" t="s">
         <v>65</v>
       </c>
-      <c r="B33" s="87"/>
-      <c r="C33" s="87">
+      <c r="B33" s="82"/>
+      <c r="C33" s="82">
         <v>1</v>
       </c>
-      <c r="D33" s="87"/>
-      <c r="E33" s="87">
+      <c r="D33" s="82"/>
+      <c r="E33" s="82">
         <v>1</v>
       </c>
-      <c r="F33" s="87">
+      <c r="F33" s="82">
         <v>0</v>
       </c>
-      <c r="G33" s="88" t="s">
+      <c r="G33" s="83" t="s">
         <v>446</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A34" s="57" t="s">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A34" s="52" t="s">
         <v>447</v>
       </c>
-      <c r="B34" s="58"/>
-      <c r="C34" s="58">
+      <c r="B34" s="53"/>
+      <c r="C34" s="53">
         <v>1</v>
       </c>
-      <c r="D34" s="58"/>
-      <c r="E34" s="58">
+      <c r="D34" s="53"/>
+      <c r="E34" s="53">
         <v>1</v>
       </c>
-      <c r="F34" s="58">
+      <c r="F34" s="53">
         <v>0</v>
       </c>
-      <c r="G34" s="59" t="s">
+      <c r="G34" s="54" t="s">
         <v>446</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A35" s="57" t="s">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A35" s="52" t="s">
         <v>70</v>
       </c>
-      <c r="B35" s="58"/>
-      <c r="C35" s="58">
+      <c r="B35" s="53"/>
+      <c r="C35" s="53">
         <v>0.01</v>
       </c>
-      <c r="D35" s="58"/>
-      <c r="E35" s="58"/>
-      <c r="F35" s="58">
+      <c r="D35" s="53"/>
+      <c r="E35" s="53"/>
+      <c r="F35" s="53">
         <v>0.2</v>
       </c>
-      <c r="G35" s="59" t="s">
+      <c r="G35" s="54" t="s">
         <v>448</v>
       </c>
     </row>
-    <row r="36" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="89" t="s">
+    <row r="36" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="84" t="s">
         <v>71</v>
       </c>
-      <c r="B36" s="58"/>
-      <c r="C36" s="58">
+      <c r="B36" s="53"/>
+      <c r="C36" s="53">
         <v>0.05</v>
       </c>
-      <c r="D36" s="58"/>
-      <c r="E36" s="58"/>
-      <c r="F36" s="58">
+      <c r="D36" s="53"/>
+      <c r="E36" s="53"/>
+      <c r="F36" s="53">
         <v>0.2</v>
       </c>
-      <c r="G36" s="59"/>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A37" s="89" t="s">
+      <c r="G36" s="54"/>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A37" s="84" t="s">
         <v>449</v>
       </c>
-      <c r="B37" s="58">
+      <c r="B37" s="53">
         <v>0.01</v>
       </c>
-      <c r="C37" s="58">
+      <c r="C37" s="53">
         <v>0.01</v>
       </c>
-      <c r="D37" s="58"/>
-      <c r="E37" s="58"/>
-      <c r="F37" s="58">
+      <c r="D37" s="53"/>
+      <c r="E37" s="53"/>
+      <c r="F37" s="53">
         <v>6.5000000000000002E-2</v>
       </c>
-      <c r="G37" s="59" t="s">
+      <c r="G37" s="54" t="s">
         <v>450</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A38" s="90" t="s">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A38" s="85" t="s">
         <v>451</v>
       </c>
-      <c r="B38" s="69">
+      <c r="B38" s="64">
         <v>0.01</v>
       </c>
-      <c r="C38" s="69">
+      <c r="C38" s="64">
         <v>0.01</v>
       </c>
-      <c r="D38" s="69"/>
-      <c r="E38" s="69">
+      <c r="D38" s="64"/>
+      <c r="E38" s="64">
         <v>0.01</v>
       </c>
-      <c r="F38" s="69">
+      <c r="F38" s="64">
         <v>6.5000000000000002E-2</v>
       </c>
-      <c r="G38" s="71" t="s">
+      <c r="G38" s="66" t="s">
         <v>452</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A39" s="57" t="s">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A39" s="52" t="s">
         <v>79</v>
       </c>
-      <c r="B39" s="58"/>
-      <c r="C39" s="58">
+      <c r="B39" s="53"/>
+      <c r="C39" s="53">
         <v>0.01</v>
       </c>
-      <c r="D39" s="58"/>
-      <c r="E39" s="58"/>
-      <c r="F39" s="58">
+      <c r="D39" s="53"/>
+      <c r="E39" s="53"/>
+      <c r="F39" s="53">
         <v>0.2</v>
       </c>
-      <c r="G39" s="59"/>
-    </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A40" s="57" t="s">
+      <c r="G39" s="54"/>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A40" s="52" t="s">
         <v>453</v>
       </c>
-      <c r="B40" s="58">
+      <c r="B40" s="53">
         <v>0.01</v>
       </c>
-      <c r="C40" s="58">
+      <c r="C40" s="53">
         <v>0.01</v>
       </c>
-      <c r="D40" s="58"/>
-      <c r="E40" s="58"/>
-      <c r="F40" s="58">
+      <c r="D40" s="53"/>
+      <c r="E40" s="53"/>
+      <c r="F40" s="53">
         <v>6.5000000000000002E-2</v>
       </c>
-      <c r="G40" s="59" t="s">
+      <c r="G40" s="54" t="s">
         <v>454</v>
       </c>
-      <c r="H40" s="91"/>
-    </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A41" s="57" t="s">
+      <c r="H40" s="86"/>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A41" s="52" t="s">
         <v>83</v>
       </c>
-      <c r="B41" s="58"/>
-      <c r="C41" s="58">
+      <c r="B41" s="53"/>
+      <c r="C41" s="53">
         <v>1</v>
       </c>
-      <c r="D41" s="58"/>
-      <c r="E41" s="58"/>
-      <c r="F41" s="58">
+      <c r="D41" s="53"/>
+      <c r="E41" s="53"/>
+      <c r="F41" s="53">
         <v>0</v>
       </c>
-      <c r="G41" s="59" t="s">
+      <c r="G41" s="54" t="s">
         <v>455</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A42" s="57" t="s">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A42" s="52" t="s">
         <v>84</v>
       </c>
-      <c r="B42" s="58">
+      <c r="B42" s="53">
         <v>3.95E-2</v>
       </c>
-      <c r="C42" s="58">
+      <c r="C42" s="53">
         <v>3.95E-2</v>
       </c>
-      <c r="D42" s="58"/>
-      <c r="E42" s="58">
+      <c r="D42" s="53"/>
+      <c r="E42" s="53">
         <v>3.95E-2</v>
       </c>
-      <c r="F42" s="58">
+      <c r="F42" s="53">
         <v>0.15</v>
       </c>
-      <c r="G42" s="59" t="s">
+      <c r="G42" s="54" t="s">
         <v>456</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A43" s="83" t="s">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A43" s="78" t="s">
         <v>457</v>
       </c>
-      <c r="B43" s="84">
+      <c r="B43" s="79">
         <v>0.01</v>
       </c>
-      <c r="C43" s="84">
+      <c r="C43" s="79">
         <v>0.01</v>
       </c>
-      <c r="D43" s="84"/>
-      <c r="E43" s="84"/>
-      <c r="F43" s="84">
+      <c r="D43" s="79"/>
+      <c r="E43" s="79"/>
+      <c r="F43" s="79">
         <v>6.5000000000000002E-2</v>
       </c>
-      <c r="G43" s="59"/>
-    </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A44" s="92" t="s">
+      <c r="G43" s="54"/>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A44" s="87" t="s">
         <v>458</v>
       </c>
-      <c r="B44" s="93">
+      <c r="B44" s="88">
         <v>0.01</v>
       </c>
-      <c r="C44" s="93" t="s">
+      <c r="C44" s="88" t="s">
         <v>459</v>
       </c>
-      <c r="D44" s="93">
+      <c r="D44" s="88">
         <v>0.01</v>
       </c>
-      <c r="E44" s="93">
+      <c r="E44" s="88">
         <v>0.01</v>
       </c>
-      <c r="F44" s="93"/>
-      <c r="G44" s="82" t="s">
+      <c r="F44" s="88"/>
+      <c r="G44" s="77" t="s">
         <v>460</v>
       </c>
     </row>
-    <row r="45" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="94" t="s">
+    <row r="45" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A45" s="89" t="s">
         <v>461</v>
       </c>
-      <c r="B45" s="95"/>
-      <c r="C45" s="95">
+      <c r="B45" s="90"/>
+      <c r="C45" s="90">
         <v>3.5000000000000003E-2</v>
       </c>
-      <c r="D45" s="95">
+      <c r="D45" s="90">
         <v>3.5000000000000003E-2</v>
       </c>
-      <c r="E45" s="95">
+      <c r="E45" s="90">
         <v>3.5000000000000003E-2</v>
       </c>
-      <c r="F45" s="95">
+      <c r="F45" s="90">
         <v>6.5000000000000002E-2</v>
       </c>
-      <c r="G45" s="96"/>
+      <c r="G45" s="91"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>